<commit_message>
Ajustes a los archivos
</commit_message>
<xml_diff>
--- a/pilar_a/data/Archivos 2025/HH_EDP_Diciembre 2025.xlsx
+++ b/pilar_a/data/Archivos 2025/HH_EDP_Diciembre 2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dacm/udd/redco_proyect/pilar_a/data/Archivos 2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEAF0A1C-8C30-A341-93F6-764F9A0D953C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04515EBC-9DCC-6C4B-B2D7-6F1B1EE1329A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B3596C6A-528B-4492-886A-86082776E7D6}"/>
+    <workbookView xWindow="-30060" yWindow="700" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B3596C6A-528B-4492-886A-86082776E7D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </externalReferences>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId5"/>
+    <pivotCache cacheId="16" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -29210,7 +29210,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9899AE29-7ED2-4D44-9AEB-CC842D073899}" name="TablaDinámica8" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9899AE29-7ED2-4D44-9AEB-CC842D073899}" name="TablaDinámica8" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:D32" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField axis="axisRow" showAll="0" sortType="descending">
@@ -100730,15 +100730,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="379e1408-2888-4c35-8838-6acad26c5d63" xsi:nil="true"/>
@@ -100747,6 +100738,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -100965,20 +100965,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50C3387C-F65F-4ABF-ABD0-FCD12BE79D2E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FCC536D1-B021-45E9-A42F-2CCF3A3CE159}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="379e1408-2888-4c35-8838-6acad26c5d63"/>
     <ds:schemaRef ds:uri="0aaa94c6-a08a-4f31-80d4-9ed0227976f0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50C3387C-F65F-4ABF-ABD0-FCD12BE79D2E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>